<commit_message>
audit pass 4: typography, grammar, decimal separators, empty cells, truncated cells, internal logs; rebuild
</commit_message>
<xml_diff>
--- a/ЛР5_Анализ_конкурентов/Excel/ЛР5_2_цифровой_товар_Левитт_Кано_TableMind.xlsx
+++ b/ЛР5_Анализ_конкурентов/Excel/ЛР5_2_цифровой_товар_Левитт_Кано_TableMind.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-89518d\ЛР5_Анализ_конкурентов\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5F7AE98-6B56-41B8-8DFC-25FB36ABA8B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B26B893-44CC-4E35-8A5E-E7BD17876EF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2205" yWindow="458" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2306" uniqueCount="1327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2306" uniqueCount="1322">
   <si>
     <t>Excel-шаблон анализа конкурентов по сайтам</t>
   </si>
@@ -3604,9 +3604,6 @@
     <t>политика конфиденциальности, условия, cookie; страницы безопасности нет</t>
   </si>
   <si>
-    <t>PerfectXL Suite: Risk Finder, Explore, Compare, Highlighter,</t>
-  </si>
-  <si>
     <t>Поиск ошибок формул и аномалий</t>
   </si>
   <si>
@@ -3685,12 +3682,6 @@
     <t>страницы продукта и принципов</t>
   </si>
   <si>
-    <t>Arixcel Explorer: логика формул, сравнение таблиц, карта фор</t>
-  </si>
-  <si>
-    <t>Model Audit, OAK (надстройка Excel), онлайн-курс по моделиро</t>
-  </si>
-  <si>
     <t>Веб-версия без установки</t>
   </si>
   <si>
@@ -3736,9 +3727,6 @@
     <t>страницы безопасности и продукта</t>
   </si>
   <si>
-    <t xml:space="preserve">FinanceOS: FP&amp;A, закрытие месяца, денежные потоки, контроль </t>
-  </si>
-  <si>
     <t>Доказательство вывода детерминированным движком</t>
   </si>
   <si>
@@ -3749,9 +3737,6 @@
   </si>
   <si>
     <t>страница интеграций</t>
-  </si>
-  <si>
-    <t xml:space="preserve">агентная автоматизация аудита, надстройка Excel, извлечение </t>
   </si>
   <si>
     <t>Извлечение данных из документов</t>
@@ -4311,7 +4296,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A414-4B5A-9EA4-A33B837B2866}"/>
+              <c16:uniqueId val="{00000000-4BA2-4D7C-9178-92BC6B3BE678}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4462,7 +4447,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3E41-4EE9-842B-76EDCA87612D}"/>
+              <c16:uniqueId val="{00000000-6E27-4A89-B93E-12C4485FB3A4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4499,7 +4484,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-3E41-4EE9-842B-76EDCA87612D}"/>
+              <c16:uniqueId val="{00000001-6E27-4A89-B93E-12C4485FB3A4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4536,7 +4521,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-3E41-4EE9-842B-76EDCA87612D}"/>
+              <c16:uniqueId val="{00000002-6E27-4A89-B93E-12C4485FB3A4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4573,7 +4558,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-3E41-4EE9-842B-76EDCA87612D}"/>
+              <c16:uniqueId val="{00000003-6E27-4A89-B93E-12C4485FB3A4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4610,7 +4595,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-3E41-4EE9-842B-76EDCA87612D}"/>
+              <c16:uniqueId val="{00000004-6E27-4A89-B93E-12C4485FB3A4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4647,7 +4632,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-3E41-4EE9-842B-76EDCA87612D}"/>
+              <c16:uniqueId val="{00000005-6E27-4A89-B93E-12C4485FB3A4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4684,7 +4669,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000006-3E41-4EE9-842B-76EDCA87612D}"/>
+              <c16:uniqueId val="{00000006-6E27-4A89-B93E-12C4485FB3A4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -10256,12 +10241,12 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="25.5">
+    <row r="7" spans="1:14" ht="51">
       <c r="A7" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>1024</v>
@@ -10270,13 +10255,13 @@
         <v>367</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>1187</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>1188</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>1189</v>
       </c>
       <c r="H7" s="2">
         <v>1</v>
@@ -10300,12 +10285,12 @@
       </c>
       <c r="N7" s="2"/>
     </row>
-    <row r="8" spans="1:14" ht="25.5">
+    <row r="8" spans="1:14" ht="51">
       <c r="A8" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>1024</v>
@@ -10314,13 +10299,13 @@
         <v>387</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>1189</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>1190</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>1191</v>
-      </c>
       <c r="G8" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H8" s="2">
         <v>1</v>
@@ -10344,12 +10329,12 @@
       </c>
       <c r="N8" s="2"/>
     </row>
-    <row r="9" spans="1:14" ht="25.5">
+    <row r="9" spans="1:14" ht="51">
       <c r="A9" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>1024</v>
@@ -10358,13 +10343,13 @@
         <v>387</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>1191</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>1192</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>1193</v>
-      </c>
       <c r="G9" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H9" s="2">
         <v>1</v>
@@ -10388,12 +10373,12 @@
       </c>
       <c r="N9" s="2"/>
     </row>
-    <row r="10" spans="1:14" ht="25.5">
+    <row r="10" spans="1:14" ht="51">
       <c r="A10" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>1024</v>
@@ -10402,13 +10387,13 @@
         <v>378</v>
       </c>
       <c r="E10" s="2" t="s">
+        <v>1193</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>1194</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>1195</v>
-      </c>
       <c r="G10" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H10" s="2">
         <v>1</v>
@@ -10432,12 +10417,12 @@
       </c>
       <c r="N10" s="2"/>
     </row>
-    <row r="11" spans="1:14" ht="25.5">
+    <row r="11" spans="1:14" ht="51">
       <c r="A11" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>1024</v>
@@ -10446,13 +10431,13 @@
         <v>374</v>
       </c>
       <c r="E11" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>1196</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>1197</v>
-      </c>
       <c r="G11" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H11" s="2">
         <v>1</v>
@@ -10476,12 +10461,12 @@
       </c>
       <c r="N11" s="2"/>
     </row>
-    <row r="12" spans="1:14" ht="25.5">
+    <row r="12" spans="1:14" ht="51">
       <c r="A12" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>1024</v>
@@ -10490,13 +10475,13 @@
         <v>378</v>
       </c>
       <c r="E12" s="2" t="s">
+        <v>1197</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>1198</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>1199</v>
-      </c>
       <c r="G12" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H12" s="2">
         <v>1</v>
@@ -10520,12 +10505,12 @@
       </c>
       <c r="N12" s="2"/>
     </row>
-    <row r="13" spans="1:14" ht="25.5">
+    <row r="13" spans="1:14" ht="51">
       <c r="A13" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>1024</v>
@@ -10534,13 +10519,13 @@
         <v>378</v>
       </c>
       <c r="E13" s="2" t="s">
+        <v>1199</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>1200</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>1201</v>
-      </c>
       <c r="G13" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H13" s="2">
         <v>1</v>
@@ -10564,12 +10549,12 @@
       </c>
       <c r="N13" s="2"/>
     </row>
-    <row r="14" spans="1:14" ht="25.5">
+    <row r="14" spans="1:14" ht="51">
       <c r="A14" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>1024</v>
@@ -10578,13 +10563,13 @@
         <v>378</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>1202</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>1203</v>
-      </c>
       <c r="G14" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H14" s="2">
         <v>1</v>
@@ -10608,12 +10593,12 @@
       </c>
       <c r="N14" s="2"/>
     </row>
-    <row r="15" spans="1:14" ht="25.5">
+    <row r="15" spans="1:14" ht="51">
       <c r="A15" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>1024</v>
@@ -10622,13 +10607,13 @@
         <v>387</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>1204</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>1205</v>
-      </c>
       <c r="G15" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H15" s="2">
         <v>1</v>
@@ -10652,12 +10637,12 @@
       </c>
       <c r="N15" s="2"/>
     </row>
-    <row r="16" spans="1:14" ht="25.5">
+    <row r="16" spans="1:14" ht="51">
       <c r="A16" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>1024</v>
@@ -10666,13 +10651,13 @@
         <v>387</v>
       </c>
       <c r="E16" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>1206</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>1207</v>
-      </c>
       <c r="G16" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H16" s="2">
         <v>1</v>
@@ -10696,12 +10681,12 @@
       </c>
       <c r="N16" s="2"/>
     </row>
-    <row r="17" spans="1:14" ht="25.5">
+    <row r="17" spans="1:14" ht="51">
       <c r="A17" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>1024</v>
@@ -10710,13 +10695,13 @@
         <v>387</v>
       </c>
       <c r="E17" s="2" t="s">
+        <v>1207</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>1208</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>1209</v>
-      </c>
       <c r="G17" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H17" s="2">
         <v>1</v>
@@ -10740,12 +10725,12 @@
       </c>
       <c r="N17" s="2"/>
     </row>
-    <row r="18" spans="1:14" ht="25.5">
+    <row r="18" spans="1:14" ht="51">
       <c r="A18" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>1024</v>
@@ -10754,13 +10739,13 @@
         <v>387</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H18" s="2">
         <v>1</v>
@@ -10784,12 +10769,12 @@
       </c>
       <c r="N18" s="2"/>
     </row>
-    <row r="19" spans="1:14" ht="25.5">
+    <row r="19" spans="1:14" ht="51">
       <c r="A19" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>1186</v>
+        <v>1029</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>1024</v>
@@ -10798,13 +10783,13 @@
         <v>387</v>
       </c>
       <c r="E19" s="2" t="s">
+        <v>1210</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>1211</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>1212</v>
-      </c>
       <c r="G19" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H19" s="2">
         <v>1</v>
@@ -10828,12 +10813,12 @@
       </c>
       <c r="N19" s="2"/>
     </row>
-    <row r="20" spans="1:14" ht="25.5">
+    <row r="20" spans="1:14" ht="38.25">
       <c r="A20" s="2" t="s">
         <v>83</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>1213</v>
+        <v>1038</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>1034</v>
@@ -10842,13 +10827,13 @@
         <v>367</v>
       </c>
       <c r="E20" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>1187</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="G20" s="2" t="s">
         <v>1188</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>1189</v>
       </c>
       <c r="H20" s="2">
         <v>1</v>
@@ -10872,12 +10857,12 @@
       </c>
       <c r="N20" s="2"/>
     </row>
-    <row r="21" spans="1:14" ht="25.5">
+    <row r="21" spans="1:14" ht="38.25">
       <c r="A21" s="2" t="s">
         <v>83</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>1213</v>
+        <v>1038</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>1034</v>
@@ -10886,13 +10871,13 @@
         <v>387</v>
       </c>
       <c r="E21" s="2" t="s">
+        <v>1189</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>1190</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>1191</v>
-      </c>
       <c r="G21" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H21" s="2">
         <v>1</v>
@@ -10916,12 +10901,12 @@
       </c>
       <c r="N21" s="2"/>
     </row>
-    <row r="22" spans="1:14" ht="25.5">
+    <row r="22" spans="1:14" ht="38.25">
       <c r="A22" s="2" t="s">
         <v>83</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>1213</v>
+        <v>1038</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>1034</v>
@@ -10930,13 +10915,13 @@
         <v>387</v>
       </c>
       <c r="E22" s="2" t="s">
+        <v>1191</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>1192</v>
       </c>
-      <c r="F22" s="2" t="s">
-        <v>1193</v>
-      </c>
       <c r="G22" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H22" s="2">
         <v>1</v>
@@ -10960,12 +10945,12 @@
       </c>
       <c r="N22" s="2"/>
     </row>
-    <row r="23" spans="1:14" ht="25.5">
+    <row r="23" spans="1:14" ht="38.25">
       <c r="A23" s="2" t="s">
         <v>83</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>1213</v>
+        <v>1038</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>1034</v>
@@ -10974,13 +10959,13 @@
         <v>374</v>
       </c>
       <c r="E23" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>1196</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>1197</v>
-      </c>
       <c r="G23" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H23" s="2">
         <v>1</v>
@@ -11004,12 +10989,12 @@
       </c>
       <c r="N23" s="2"/>
     </row>
-    <row r="24" spans="1:14" ht="25.5">
+    <row r="24" spans="1:14" ht="38.25">
       <c r="A24" s="2" t="s">
         <v>83</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>1213</v>
+        <v>1038</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>1034</v>
@@ -11018,13 +11003,13 @@
         <v>387</v>
       </c>
       <c r="E24" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>1204</v>
       </c>
-      <c r="F24" s="2" t="s">
-        <v>1205</v>
-      </c>
       <c r="G24" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H24" s="2">
         <v>1</v>
@@ -11048,12 +11033,12 @@
       </c>
       <c r="N24" s="2"/>
     </row>
-    <row r="25" spans="1:14" ht="25.5">
+    <row r="25" spans="1:14" ht="38.25">
       <c r="A25" s="2" t="s">
         <v>83</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>1213</v>
+        <v>1038</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>1034</v>
@@ -11062,13 +11047,13 @@
         <v>387</v>
       </c>
       <c r="E25" s="2" t="s">
+        <v>1207</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>1208</v>
       </c>
-      <c r="F25" s="2" t="s">
-        <v>1209</v>
-      </c>
       <c r="G25" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H25" s="2">
         <v>1</v>
@@ -11092,12 +11077,12 @@
       </c>
       <c r="N25" s="2"/>
     </row>
-    <row r="26" spans="1:14" ht="25.5">
+    <row r="26" spans="1:14" ht="38.25">
       <c r="A26" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>1214</v>
+        <v>1044</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>1040</v>
@@ -11106,13 +11091,13 @@
         <v>367</v>
       </c>
       <c r="E26" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>1187</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>1188</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>1189</v>
       </c>
       <c r="H26" s="2">
         <v>1</v>
@@ -11136,12 +11121,12 @@
       </c>
       <c r="N26" s="2"/>
     </row>
-    <row r="27" spans="1:14" ht="25.5">
+    <row r="27" spans="1:14" ht="38.25">
       <c r="A27" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>1214</v>
+        <v>1044</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>1040</v>
@@ -11150,13 +11135,13 @@
         <v>387</v>
       </c>
       <c r="E27" s="2" t="s">
+        <v>1189</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>1190</v>
       </c>
-      <c r="F27" s="2" t="s">
-        <v>1191</v>
-      </c>
       <c r="G27" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H27" s="2">
         <v>1</v>
@@ -11180,12 +11165,12 @@
       </c>
       <c r="N27" s="2"/>
     </row>
-    <row r="28" spans="1:14" ht="25.5">
+    <row r="28" spans="1:14" ht="38.25">
       <c r="A28" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>1214</v>
+        <v>1044</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>1040</v>
@@ -11194,13 +11179,13 @@
         <v>378</v>
       </c>
       <c r="E28" s="2" t="s">
+        <v>1193</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>1194</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>1195</v>
-      </c>
       <c r="G28" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H28" s="2">
         <v>1</v>
@@ -11224,12 +11209,12 @@
       </c>
       <c r="N28" s="2"/>
     </row>
-    <row r="29" spans="1:14" ht="25.5">
+    <row r="29" spans="1:14" ht="38.25">
       <c r="A29" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>1214</v>
+        <v>1044</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>1040</v>
@@ -11238,13 +11223,13 @@
         <v>374</v>
       </c>
       <c r="E29" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>1196</v>
       </c>
-      <c r="F29" s="2" t="s">
-        <v>1197</v>
-      </c>
       <c r="G29" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H29" s="2">
         <v>1</v>
@@ -11268,12 +11253,12 @@
       </c>
       <c r="N29" s="2"/>
     </row>
-    <row r="30" spans="1:14" ht="25.5">
+    <row r="30" spans="1:14" ht="38.25">
       <c r="A30" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>1214</v>
+        <v>1044</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>1040</v>
@@ -11282,13 +11267,13 @@
         <v>378</v>
       </c>
       <c r="E30" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>1202</v>
       </c>
-      <c r="F30" s="2" t="s">
-        <v>1203</v>
-      </c>
       <c r="G30" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H30" s="2">
         <v>1</v>
@@ -11312,12 +11297,12 @@
       </c>
       <c r="N30" s="2"/>
     </row>
-    <row r="31" spans="1:14" ht="25.5">
+    <row r="31" spans="1:14" ht="38.25">
       <c r="A31" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>1214</v>
+        <v>1044</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>1040</v>
@@ -11326,13 +11311,13 @@
         <v>387</v>
       </c>
       <c r="E31" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>1204</v>
       </c>
-      <c r="F31" s="2" t="s">
-        <v>1205</v>
-      </c>
       <c r="G31" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H31" s="2">
         <v>1</v>
@@ -11356,12 +11341,12 @@
       </c>
       <c r="N31" s="2"/>
     </row>
-    <row r="32" spans="1:14" ht="25.5">
+    <row r="32" spans="1:14" ht="38.25">
       <c r="A32" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>1214</v>
+        <v>1044</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>1040</v>
@@ -11370,13 +11355,13 @@
         <v>387</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H32" s="2">
         <v>1</v>
@@ -11400,12 +11385,12 @@
       </c>
       <c r="N32" s="2"/>
     </row>
-    <row r="33" spans="1:14" ht="25.5">
+    <row r="33" spans="1:14" ht="38.25">
       <c r="A33" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>1214</v>
+        <v>1044</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>1040</v>
@@ -11414,13 +11399,13 @@
         <v>387</v>
       </c>
       <c r="E33" s="2" t="s">
+        <v>1210</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>1211</v>
       </c>
-      <c r="F33" s="2" t="s">
-        <v>1212</v>
-      </c>
       <c r="G33" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H33" s="2">
         <v>1</v>
@@ -11458,13 +11443,13 @@
         <v>387</v>
       </c>
       <c r="E34" s="2" t="s">
+        <v>1189</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>1190</v>
       </c>
-      <c r="F34" s="2" t="s">
-        <v>1191</v>
-      </c>
       <c r="G34" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H34" s="2">
         <v>1</v>
@@ -11502,13 +11487,13 @@
         <v>374</v>
       </c>
       <c r="E35" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>1196</v>
       </c>
-      <c r="F35" s="2" t="s">
-        <v>1197</v>
-      </c>
       <c r="G35" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H35" s="2">
         <v>1</v>
@@ -11546,13 +11531,13 @@
         <v>374</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>1215</v>
+        <v>1212</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>1070</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H36" s="2">
         <v>1</v>
@@ -11590,13 +11575,13 @@
         <v>387</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>1217</v>
+        <v>1214</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H37" s="2">
         <v>1</v>
@@ -11634,13 +11619,13 @@
         <v>378</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>1218</v>
+        <v>1215</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H38" s="2">
         <v>1</v>
@@ -11678,13 +11663,13 @@
         <v>378</v>
       </c>
       <c r="E39" s="2" t="s">
+        <v>1197</v>
+      </c>
+      <c r="F39" s="2" t="s">
         <v>1198</v>
       </c>
-      <c r="F39" s="2" t="s">
-        <v>1199</v>
-      </c>
       <c r="G39" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H39" s="2">
         <v>1</v>
@@ -11722,13 +11707,13 @@
         <v>378</v>
       </c>
       <c r="E40" s="2" t="s">
+        <v>1199</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>1200</v>
       </c>
-      <c r="F40" s="2" t="s">
-        <v>1201</v>
-      </c>
       <c r="G40" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H40" s="2">
         <v>1</v>
@@ -11766,13 +11751,13 @@
         <v>387</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>1220</v>
+        <v>1217</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>1133</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H41" s="2">
         <v>1</v>
@@ -11810,13 +11795,13 @@
         <v>378</v>
       </c>
       <c r="E42" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>1202</v>
       </c>
-      <c r="F42" s="2" t="s">
-        <v>1203</v>
-      </c>
       <c r="G42" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H42" s="2">
         <v>1</v>
@@ -11854,13 +11839,13 @@
         <v>387</v>
       </c>
       <c r="E43" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>1206</v>
       </c>
-      <c r="F43" s="2" t="s">
-        <v>1207</v>
-      </c>
       <c r="G43" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H43" s="2">
         <v>1</v>
@@ -11898,13 +11883,13 @@
         <v>393</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>1221</v>
+        <v>1218</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>1222</v>
+        <v>1219</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H44" s="2">
         <v>1</v>
@@ -11942,13 +11927,13 @@
         <v>387</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>1223</v>
+        <v>1220</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H45" s="2">
         <v>1</v>
@@ -11986,13 +11971,13 @@
         <v>378</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>1225</v>
+        <v>1222</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H46" s="2">
         <v>1</v>
@@ -12030,13 +12015,13 @@
         <v>387</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>1227</v>
+        <v>1224</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H47" s="2">
         <v>1</v>
@@ -12074,13 +12059,13 @@
         <v>393</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>1228</v>
+        <v>1225</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>1229</v>
+        <v>1226</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H48" s="2">
         <v>1</v>
@@ -12118,13 +12103,13 @@
         <v>374</v>
       </c>
       <c r="E49" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="F49" s="2" t="s">
         <v>1196</v>
       </c>
-      <c r="F49" s="2" t="s">
-        <v>1197</v>
-      </c>
       <c r="G49" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H49" s="2">
         <v>1</v>
@@ -12162,13 +12147,13 @@
         <v>374</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>1215</v>
+        <v>1212</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>1070</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H50" s="2">
         <v>1</v>
@@ -12206,13 +12191,13 @@
         <v>387</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>1217</v>
+        <v>1214</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H51" s="2">
         <v>1</v>
@@ -12250,13 +12235,13 @@
         <v>378</v>
       </c>
       <c r="E52" s="2" t="s">
+        <v>1197</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>1198</v>
       </c>
-      <c r="F52" s="2" t="s">
-        <v>1199</v>
-      </c>
       <c r="G52" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H52" s="2">
         <v>1</v>
@@ -12294,13 +12279,13 @@
         <v>378</v>
       </c>
       <c r="E53" s="2" t="s">
+        <v>1199</v>
+      </c>
+      <c r="F53" s="2" t="s">
         <v>1200</v>
       </c>
-      <c r="F53" s="2" t="s">
-        <v>1201</v>
-      </c>
       <c r="G53" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H53" s="2">
         <v>1</v>
@@ -12338,13 +12323,13 @@
         <v>387</v>
       </c>
       <c r="E54" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="F54" s="2" t="s">
         <v>1204</v>
       </c>
-      <c r="F54" s="2" t="s">
-        <v>1205</v>
-      </c>
       <c r="G54" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H54" s="2">
         <v>1</v>
@@ -12382,13 +12367,13 @@
         <v>387</v>
       </c>
       <c r="E55" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="F55" s="2" t="s">
         <v>1206</v>
       </c>
-      <c r="F55" s="2" t="s">
-        <v>1207</v>
-      </c>
       <c r="G55" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H55" s="2">
         <v>1</v>
@@ -12426,13 +12411,13 @@
         <v>387</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>1223</v>
+        <v>1220</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H56" s="2">
         <v>1</v>
@@ -12461,7 +12446,7 @@
         <v>87</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>1059</v>
@@ -12470,13 +12455,13 @@
         <v>378</v>
       </c>
       <c r="E57" s="2" t="s">
+        <v>1193</v>
+      </c>
+      <c r="F57" s="2" t="s">
         <v>1194</v>
       </c>
-      <c r="F57" s="2" t="s">
-        <v>1195</v>
-      </c>
       <c r="G57" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H57" s="2">
         <v>1</v>
@@ -12505,7 +12490,7 @@
         <v>87</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>1059</v>
@@ -12514,13 +12499,13 @@
         <v>374</v>
       </c>
       <c r="E58" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="F58" s="2" t="s">
         <v>1196</v>
       </c>
-      <c r="F58" s="2" t="s">
-        <v>1197</v>
-      </c>
       <c r="G58" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H58" s="2">
         <v>1</v>
@@ -12549,7 +12534,7 @@
         <v>87</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>1059</v>
@@ -12558,13 +12543,13 @@
         <v>374</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>1215</v>
+        <v>1212</v>
       </c>
       <c r="F59" s="2" t="s">
         <v>1070</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H59" s="2">
         <v>1</v>
@@ -12593,7 +12578,7 @@
         <v>87</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>1059</v>
@@ -12602,13 +12587,13 @@
         <v>387</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>1217</v>
+        <v>1214</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H60" s="2">
         <v>1</v>
@@ -12637,7 +12622,7 @@
         <v>87</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>1059</v>
@@ -12646,13 +12631,13 @@
         <v>393</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>1231</v>
+        <v>1227</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>1232</v>
+        <v>1228</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H61" s="2">
         <v>1</v>
@@ -12681,7 +12666,7 @@
         <v>87</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>1059</v>
@@ -12690,13 +12675,13 @@
         <v>378</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>1218</v>
+        <v>1215</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H62" s="2">
         <v>1</v>
@@ -12725,7 +12710,7 @@
         <v>87</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>1059</v>
@@ -12734,13 +12719,13 @@
         <v>387</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>1220</v>
+        <v>1217</v>
       </c>
       <c r="F63" s="2" t="s">
         <v>1133</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H63" s="2">
         <v>1</v>
@@ -12769,7 +12754,7 @@
         <v>87</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>1059</v>
@@ -12778,13 +12763,13 @@
         <v>378</v>
       </c>
       <c r="E64" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="F64" s="2" t="s">
         <v>1202</v>
       </c>
-      <c r="F64" s="2" t="s">
-        <v>1203</v>
-      </c>
       <c r="G64" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H64" s="2">
         <v>1</v>
@@ -12813,7 +12798,7 @@
         <v>87</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>1059</v>
@@ -12822,13 +12807,13 @@
         <v>387</v>
       </c>
       <c r="E65" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="F65" s="2" t="s">
         <v>1204</v>
       </c>
-      <c r="F65" s="2" t="s">
-        <v>1205</v>
-      </c>
       <c r="G65" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H65" s="2">
         <v>1</v>
@@ -12857,7 +12842,7 @@
         <v>87</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>1059</v>
@@ -12866,13 +12851,13 @@
         <v>387</v>
       </c>
       <c r="E66" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="F66" s="2" t="s">
         <v>1206</v>
       </c>
-      <c r="F66" s="2" t="s">
-        <v>1207</v>
-      </c>
       <c r="G66" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H66" s="2">
         <v>1</v>
@@ -12901,7 +12886,7 @@
         <v>87</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>1059</v>
@@ -12910,13 +12895,13 @@
         <v>387</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>1223</v>
+        <v>1220</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H67" s="2">
         <v>1</v>
@@ -12945,7 +12930,7 @@
         <v>87</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C68" s="2" t="s">
         <v>1059</v>
@@ -12954,13 +12939,13 @@
         <v>393</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>1233</v>
+        <v>1229</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>1234</v>
+        <v>1230</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H68" s="2">
         <v>1</v>
@@ -12989,7 +12974,7 @@
         <v>87</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>1059</v>
@@ -12998,13 +12983,13 @@
         <v>378</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>1225</v>
+        <v>1222</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H69" s="2">
         <v>1</v>
@@ -13033,7 +13018,7 @@
         <v>87</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>1230</v>
+        <v>1063</v>
       </c>
       <c r="C70" s="2" t="s">
         <v>1059</v>
@@ -13042,13 +13027,13 @@
         <v>387</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>1227</v>
+        <v>1224</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H70" s="2">
         <v>1</v>
@@ -13072,12 +13057,12 @@
       </c>
       <c r="N70" s="2"/>
     </row>
-    <row r="71" spans="1:14" ht="25.5">
+    <row r="71" spans="1:14" ht="38.25">
       <c r="A71" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>1065</v>
@@ -13086,13 +13071,13 @@
         <v>378</v>
       </c>
       <c r="E71" s="2" t="s">
+        <v>1193</v>
+      </c>
+      <c r="F71" s="2" t="s">
         <v>1194</v>
       </c>
-      <c r="F71" s="2" t="s">
-        <v>1195</v>
-      </c>
       <c r="G71" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H71" s="2">
         <v>1</v>
@@ -13116,12 +13101,12 @@
       </c>
       <c r="N71" s="2"/>
     </row>
-    <row r="72" spans="1:14" ht="25.5">
+    <row r="72" spans="1:14" ht="38.25">
       <c r="A72" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C72" s="2" t="s">
         <v>1065</v>
@@ -13130,13 +13115,13 @@
         <v>374</v>
       </c>
       <c r="E72" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="F72" s="2" t="s">
         <v>1196</v>
       </c>
-      <c r="F72" s="2" t="s">
-        <v>1197</v>
-      </c>
       <c r="G72" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H72" s="2">
         <v>1</v>
@@ -13160,12 +13145,12 @@
       </c>
       <c r="N72" s="2"/>
     </row>
-    <row r="73" spans="1:14" ht="25.5">
+    <row r="73" spans="1:14" ht="38.25">
       <c r="A73" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C73" s="2" t="s">
         <v>1065</v>
@@ -13174,13 +13159,13 @@
         <v>374</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>1215</v>
+        <v>1212</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>1070</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H73" s="2">
         <v>1</v>
@@ -13204,12 +13189,12 @@
       </c>
       <c r="N73" s="2"/>
     </row>
-    <row r="74" spans="1:14" ht="25.5">
+    <row r="74" spans="1:14" ht="38.25">
       <c r="A74" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C74" s="2" t="s">
         <v>1065</v>
@@ -13218,13 +13203,13 @@
         <v>387</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>1217</v>
+        <v>1214</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H74" s="2">
         <v>1</v>
@@ -13248,12 +13233,12 @@
       </c>
       <c r="N74" s="2"/>
     </row>
-    <row r="75" spans="1:14" ht="25.5">
+    <row r="75" spans="1:14" ht="38.25">
       <c r="A75" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C75" s="2" t="s">
         <v>1065</v>
@@ -13262,13 +13247,13 @@
         <v>393</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>1231</v>
+        <v>1227</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>1232</v>
+        <v>1228</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H75" s="2">
         <v>1</v>
@@ -13292,12 +13277,12 @@
       </c>
       <c r="N75" s="2"/>
     </row>
-    <row r="76" spans="1:14" ht="25.5">
+    <row r="76" spans="1:14" ht="38.25">
       <c r="A76" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>1065</v>
@@ -13306,13 +13291,13 @@
         <v>378</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>1218</v>
+        <v>1215</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H76" s="2">
         <v>1</v>
@@ -13336,12 +13321,12 @@
       </c>
       <c r="N76" s="2"/>
     </row>
-    <row r="77" spans="1:14" ht="25.5">
+    <row r="77" spans="1:14" ht="38.25">
       <c r="A77" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>1065</v>
@@ -13350,13 +13335,13 @@
         <v>387</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>1220</v>
+        <v>1217</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>1133</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H77" s="2">
         <v>1</v>
@@ -13380,12 +13365,12 @@
       </c>
       <c r="N77" s="2"/>
     </row>
-    <row r="78" spans="1:14" ht="25.5">
+    <row r="78" spans="1:14" ht="38.25">
       <c r="A78" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>1065</v>
@@ -13394,13 +13379,13 @@
         <v>378</v>
       </c>
       <c r="E78" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="F78" s="2" t="s">
         <v>1202</v>
       </c>
-      <c r="F78" s="2" t="s">
-        <v>1203</v>
-      </c>
       <c r="G78" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H78" s="2">
         <v>1</v>
@@ -13424,12 +13409,12 @@
       </c>
       <c r="N78" s="2"/>
     </row>
-    <row r="79" spans="1:14" ht="25.5">
+    <row r="79" spans="1:14" ht="38.25">
       <c r="A79" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>1065</v>
@@ -13438,13 +13423,13 @@
         <v>387</v>
       </c>
       <c r="E79" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="F79" s="2" t="s">
         <v>1204</v>
       </c>
-      <c r="F79" s="2" t="s">
-        <v>1205</v>
-      </c>
       <c r="G79" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H79" s="2">
         <v>1</v>
@@ -13468,12 +13453,12 @@
       </c>
       <c r="N79" s="2"/>
     </row>
-    <row r="80" spans="1:14" ht="25.5">
+    <row r="80" spans="1:14" ht="38.25">
       <c r="A80" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>1065</v>
@@ -13482,13 +13467,13 @@
         <v>387</v>
       </c>
       <c r="E80" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="F80" s="2" t="s">
         <v>1206</v>
       </c>
-      <c r="F80" s="2" t="s">
-        <v>1207</v>
-      </c>
       <c r="G80" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H80" s="2">
         <v>1</v>
@@ -13512,12 +13497,12 @@
       </c>
       <c r="N80" s="2"/>
     </row>
-    <row r="81" spans="1:14" ht="25.5">
+    <row r="81" spans="1:14" ht="38.25">
       <c r="A81" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>1065</v>
@@ -13526,13 +13511,13 @@
         <v>393</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>1233</v>
+        <v>1229</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>1234</v>
+        <v>1230</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H81" s="2">
         <v>1</v>
@@ -13556,12 +13541,12 @@
       </c>
       <c r="N81" s="2"/>
     </row>
-    <row r="82" spans="1:14" ht="25.5">
+    <row r="82" spans="1:14" ht="38.25">
       <c r="A82" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>1065</v>
@@ -13570,13 +13555,13 @@
         <v>378</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>1225</v>
+        <v>1222</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H82" s="2">
         <v>1</v>
@@ -13600,12 +13585,12 @@
       </c>
       <c r="N82" s="2"/>
     </row>
-    <row r="83" spans="1:14" ht="25.5">
+    <row r="83" spans="1:14" ht="38.25">
       <c r="A83" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>1065</v>
@@ -13614,13 +13599,13 @@
         <v>393</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>1228</v>
+        <v>1225</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>1229</v>
+        <v>1226</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H83" s="2">
         <v>1</v>
@@ -13644,12 +13629,12 @@
       </c>
       <c r="N83" s="2"/>
     </row>
-    <row r="84" spans="1:14" ht="25.5">
+    <row r="84" spans="1:14" ht="38.25">
       <c r="A84" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>1235</v>
+        <v>1068</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>1065</v>
@@ -13658,13 +13643,13 @@
         <v>393</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>1236</v>
+        <v>1231</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="H84" s="2">
         <v>1</v>
@@ -18708,13 +18693,13 @@
         <v>152</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>1232</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>1187</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>1237</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>1188</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>375</v>
@@ -18737,7 +18722,7 @@
         <v>Потенциальный обязательный разрыв</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>1238</v>
+        <v>1233</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
@@ -18747,13 +18732,13 @@
         <v>153</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>1234</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>1190</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>1239</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>1191</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>371</v>
@@ -18776,7 +18761,7 @@
         <v>Конкурентная норма с влиянием на выбор</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>1240</v>
+        <v>1235</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
@@ -18786,13 +18771,13 @@
         <v>154</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>1191</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>1236</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>1192</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>1241</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>1193</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>371</v>
@@ -18815,7 +18800,7 @@
         <v>Зона усиления ценности</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>1242</v>
+        <v>1237</v>
       </c>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
@@ -18825,13 +18810,13 @@
         <v>155</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>1238</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>1194</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>1243</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>1195</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>371</v>
@@ -18854,7 +18839,7 @@
         <v>Конкурентная норма с влиянием на выбор</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>1244</v>
+        <v>1239</v>
       </c>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
@@ -18864,13 +18849,13 @@
         <v>156</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>1240</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>1196</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>1245</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>1197</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>375</v>
@@ -18893,7 +18878,7 @@
         <v>Минимальный рыночный стандарт</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>1246</v>
+        <v>1241</v>
       </c>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
@@ -18903,10 +18888,10 @@
         <v>157</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1215</v>
+        <v>1212</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1247</v>
+        <v>1242</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>1070</v>
@@ -18932,7 +18917,7 @@
         <v>Переходит в ожидаемую норму</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>1248</v>
+        <v>1243</v>
       </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
@@ -18942,13 +18927,13 @@
         <v>158</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>1249</v>
+        <v>1244</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>1217</v>
+        <v>1214</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>394</v>
@@ -18971,7 +18956,7 @@
         <v>Переходит в ожидаемую норму</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>1250</v>
+        <v>1245</v>
       </c>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
@@ -18981,13 +18966,13 @@
         <v>159</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1231</v>
+        <v>1227</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1251</v>
+        <v>1246</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>1232</v>
+        <v>1228</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>394</v>
@@ -19010,7 +18995,7 @@
         <v>Зона дифференциации</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>1252</v>
+        <v>1247</v>
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
@@ -19020,13 +19005,13 @@
         <v>160</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>1218</v>
+        <v>1215</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>1253</v>
+        <v>1248</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>375</v>
@@ -19049,7 +19034,7 @@
         <v>Потенциальный обязательный разрыв</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>1254</v>
+        <v>1249</v>
       </c>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
@@ -19059,13 +19044,13 @@
         <v>161</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>1197</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>1250</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>1198</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>1255</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>1199</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>375</v>
@@ -19088,7 +19073,7 @@
         <v>Потенциальный обязательный разрыв</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>1256</v>
+        <v>1251</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
@@ -19098,13 +19083,13 @@
         <v>162</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>1252</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>1200</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>1257</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>1201</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>371</v>
@@ -19127,7 +19112,7 @@
         <v>Зона усиления ценности</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>1258</v>
+        <v>1253</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
@@ -19137,10 +19122,10 @@
         <v>163</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1220</v>
+        <v>1217</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1259</v>
+        <v>1254</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>1133</v>
@@ -19166,7 +19151,7 @@
         <v>Зона усиления ценности</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>1260</v>
+        <v>1255</v>
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
@@ -19176,13 +19161,13 @@
         <v>164</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>1256</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>1202</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>1261</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>1203</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>371</v>
@@ -19205,7 +19190,7 @@
         <v>Конкурентная норма с влиянием на выбор</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>1262</v>
+        <v>1257</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
@@ -19215,13 +19200,13 @@
         <v>165</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>1258</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>1204</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>1263</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>1205</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>970</v>
@@ -19244,7 +19229,7 @@
         <v>Не делать при дефиците ресурсов</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>1264</v>
+        <v>1259</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
@@ -19254,13 +19239,13 @@
         <v>166</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>1260</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>1206</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>1265</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>1207</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>371</v>
@@ -19283,7 +19268,7 @@
         <v>Конкурентная норма с влиянием на выбор</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>1266</v>
+        <v>1261</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
@@ -19293,13 +19278,13 @@
         <v>167</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>1221</v>
+        <v>1218</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1267</v>
+        <v>1262</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>1222</v>
+        <v>1219</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>394</v>
@@ -19322,7 +19307,7 @@
         <v>Зона дифференциации</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>1242</v>
+        <v>1237</v>
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
@@ -19332,13 +19317,13 @@
         <v>168</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>1207</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>1263</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>1208</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>1268</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>1209</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>371</v>
@@ -19361,7 +19346,7 @@
         <v>Зона усиления ценности</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>1269</v>
+        <v>1264</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
@@ -19371,13 +19356,13 @@
         <v>169</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1270</v>
+        <v>1265</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>394</v>
@@ -19400,7 +19385,7 @@
         <v>Зона дифференциации</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>1269</v>
+        <v>1264</v>
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
@@ -19410,13 +19395,13 @@
         <v>170</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>1210</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>1266</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>1211</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>1271</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>1212</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>371</v>
@@ -19439,7 +19424,7 @@
         <v>Зона усиления ценности</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>1272</v>
+        <v>1267</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
@@ -19449,13 +19434,13 @@
         <v>171</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>1223</v>
+        <v>1220</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1273</v>
+        <v>1268</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>970</v>
@@ -19478,7 +19463,7 @@
         <v>Не делать при дефиците ресурсов</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>1274</v>
+        <v>1269</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
@@ -19488,13 +19473,13 @@
         <v>172</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>1233</v>
+        <v>1229</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>1275</v>
+        <v>1270</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>1234</v>
+        <v>1230</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>970</v>
@@ -19517,7 +19502,7 @@
         <v>Не делать при дефиците ресурсов</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>1276</v>
+        <v>1271</v>
       </c>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
@@ -19527,13 +19512,13 @@
         <v>173</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>1225</v>
+        <v>1222</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>1277</v>
+        <v>1272</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>375</v>
@@ -19556,7 +19541,7 @@
         <v>Потенциальный обязательный разрыв</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>1254</v>
+        <v>1249</v>
       </c>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
@@ -19566,13 +19551,13 @@
         <v>174</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>1278</v>
+        <v>1273</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>1227</v>
+        <v>1224</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>371</v>
@@ -19595,7 +19580,7 @@
         <v>Зона усиления ценности</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>1279</v>
+        <v>1274</v>
       </c>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
@@ -19605,13 +19590,13 @@
         <v>175</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>1228</v>
+        <v>1225</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>1280</v>
+        <v>1275</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>1229</v>
+        <v>1226</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>371</v>
@@ -19634,7 +19619,7 @@
         <v>Зона усиления ценности</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>1269</v>
+        <v>1264</v>
       </c>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
@@ -19644,13 +19629,13 @@
         <v>176</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>1236</v>
+        <v>1231</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>1281</v>
+        <v>1276</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>970</v>
@@ -19673,7 +19658,7 @@
         <v>Не делать при дефиците ресурсов</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>1276</v>
+        <v>1271</v>
       </c>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
@@ -23860,10 +23845,10 @@
         <v>366</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1305</v>
+        <v>1300</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1306</v>
+        <v>1301</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>367</v>
@@ -23886,10 +23871,10 @@
         <v>370</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1307</v>
+        <v>1302</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1308</v>
+        <v>1303</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>367</v>
@@ -23912,10 +23897,10 @@
         <v>373</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1309</v>
+        <v>1304</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1310</v>
+        <v>1305</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>374</v>
@@ -23938,10 +23923,10 @@
         <v>377</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1311</v>
+        <v>1306</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>1312</v>
+        <v>1307</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>378</v>
@@ -23964,10 +23949,10 @@
         <v>380</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>1313</v>
+        <v>1308</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>1310</v>
+        <v>1305</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>378</v>
@@ -23990,10 +23975,10 @@
         <v>382</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1314</v>
+        <v>1309</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>1315</v>
+        <v>1310</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>378</v>
@@ -24016,7 +24001,7 @@
         <v>384</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>1316</v>
+        <v>1311</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>165</v>
@@ -24042,10 +24027,10 @@
         <v>386</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1317</v>
+        <v>1312</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>1318</v>
+        <v>1313</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>387</v>
@@ -24068,10 +24053,10 @@
         <v>390</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>1319</v>
+        <v>1314</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>1320</v>
+        <v>1315</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>387</v>
@@ -24094,10 +24079,10 @@
         <v>392</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1321</v>
+        <v>1316</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>1322</v>
+        <v>1317</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>393</v>
@@ -24120,10 +24105,10 @@
         <v>396</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>1323</v>
+        <v>1318</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>1324</v>
+        <v>1319</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>397</v>
@@ -24146,10 +24131,10 @@
         <v>400</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1325</v>
+        <v>1320</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>1326</v>
+        <v>1321</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>401</v>
@@ -27814,10 +27799,10 @@
         <v>537</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>367</v>
@@ -27848,10 +27833,10 @@
         <v>538</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>387</v>
@@ -27882,10 +27867,10 @@
         <v>539</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>387</v>
@@ -27916,10 +27901,10 @@
         <v>540</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>378</v>
@@ -27950,10 +27935,10 @@
         <v>541</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>374</v>
@@ -27984,10 +27969,10 @@
         <v>542</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1215</v>
+        <v>1212</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>374</v>
@@ -28018,10 +28003,10 @@
         <v>543</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>387</v>
@@ -28052,10 +28037,10 @@
         <v>544</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1231</v>
+        <v>1227</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>393</v>
@@ -28086,10 +28071,10 @@
         <v>545</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>1218</v>
+        <v>1215</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>378</v>
@@ -28120,10 +28105,10 @@
         <v>546</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>378</v>
@@ -28154,10 +28139,10 @@
         <v>547</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>378</v>
@@ -28188,10 +28173,10 @@
         <v>548</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1220</v>
+        <v>1217</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>387</v>
@@ -28222,10 +28207,10 @@
         <v>549</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>378</v>
@@ -28256,10 +28241,10 @@
         <v>550</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>387</v>
@@ -28290,10 +28275,10 @@
         <v>551</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>387</v>
@@ -28324,10 +28309,10 @@
         <v>552</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>1221</v>
+        <v>1218</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>393</v>
@@ -28358,10 +28343,10 @@
         <v>553</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>387</v>
@@ -28392,10 +28377,10 @@
         <v>554</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>387</v>
@@ -28426,10 +28411,10 @@
         <v>555</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>387</v>
@@ -28460,10 +28445,10 @@
         <v>556</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>1223</v>
+        <v>1220</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>387</v>
@@ -28494,10 +28479,10 @@
         <v>557</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>1233</v>
+        <v>1229</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>393</v>
@@ -28528,10 +28513,10 @@
         <v>558</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>1225</v>
+        <v>1222</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>378</v>
@@ -28562,10 +28547,10 @@
         <v>559</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>387</v>
@@ -28596,10 +28581,10 @@
         <v>560</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>1228</v>
+        <v>1225</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>393</v>
@@ -28630,10 +28615,10 @@
         <v>561</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>1236</v>
+        <v>1231</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>393</v>
@@ -32678,10 +32663,10 @@
         <v>81</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1283</v>
+        <v>1278</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1284</v>
+        <v>1279</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -32709,7 +32694,7 @@
         <v>Потенциальное преимущество</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>1285</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="25.5">
@@ -32720,15 +32705,15 @@
         <v>81</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1286</v>
+        <v>1281</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1287</v>
+        <v>1282</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2" t="s">
-        <v>1288</v>
+        <v>1283</v>
       </c>
       <c r="H8" s="2">
         <v>3</v>
@@ -32751,7 +32736,7 @@
         <v>Потенциальное преимущество</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>1285</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="25.5">
@@ -32762,15 +32747,15 @@
         <v>85</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1289</v>
+        <v>1284</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1290</v>
+        <v>1285</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
-        <v>1291</v>
+        <v>1286</v>
       </c>
       <c r="H9" s="2">
         <v>2</v>
@@ -32793,7 +32778,7 @@
         <v>Потенциальное преимущество</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>1285</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="25.5">
@@ -32804,10 +32789,10 @@
         <v>85</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1292</v>
+        <v>1287</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>1293</v>
+        <v>1288</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -32835,7 +32820,7 @@
         <v>Сильное преимущество</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>1285</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="25.5">
@@ -32846,15 +32831,15 @@
         <v>86</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>1294</v>
+        <v>1289</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>1295</v>
+        <v>1290</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
-        <v>1296</v>
+        <v>1291</v>
       </c>
       <c r="H11" s="2">
         <v>1</v>
@@ -32877,7 +32862,7 @@
         <v>Слабое преимущество</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>1285</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="25.5">
@@ -32888,15 +32873,15 @@
         <v>87</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1297</v>
+        <v>1292</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>1298</v>
+        <v>1293</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
-        <v>1299</v>
+        <v>1294</v>
       </c>
       <c r="H12" s="2">
         <v>4</v>
@@ -32919,7 +32904,7 @@
         <v>Сильное преимущество</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>1285</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="25.5">
@@ -32930,10 +32915,10 @@
         <v>88</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>1300</v>
+        <v>1295</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>1301</v>
+        <v>1296</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
@@ -32961,7 +32946,7 @@
         <v>Сильное преимущество</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>1285</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="25.5">
@@ -32972,15 +32957,15 @@
         <v>84</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1302</v>
+        <v>1297</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>1303</v>
+        <v>1298</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2" t="s">
-        <v>1304</v>
+        <v>1299</v>
       </c>
       <c r="H14" s="2">
         <v>5</v>
@@ -33003,7 +32988,7 @@
         <v>Потенциальное преимущество</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>1285</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="15" spans="1:14">

</xml_diff>